<commit_message>
Covert DevOps to Linux/Bash
</commit_message>
<xml_diff>
--- a/SBC6502 Bus.xlsx
+++ b/SBC6502 Bus.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29328"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29426"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="H:\_cwg-base__Home\Computer Archtecture\Retro Computing\SBC6502\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9D8EE3BE-053B-496C-AFF5-0DD5DE82B42F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{124E461A-43F9-4FAE-AA91-D9ED67712699}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-16305" yWindow="9210" windowWidth="16410" windowHeight="14145" xr2:uid="{07605504-F6D8-4284-A17B-5B2F32B70D70}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="15720" xr2:uid="{07605504-F6D8-4284-A17B-5B2F32B70D70}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -771,7 +771,6 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CF3C1C7E-605D-41A8-B4C8-47EE79D051C7}">
-  <sheetPr filterMode="1"/>
   <dimension ref="A1:L108"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
@@ -1016,7 +1015,7 @@
       </c>
       <c r="K9" s="1"/>
     </row>
-    <row r="10" spans="1:12" hidden="1" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A10">
         <v>8</v>
       </c>
@@ -1036,7 +1035,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="11" spans="1:12" hidden="1" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A11">
         <v>9</v>
       </c>
@@ -1071,7 +1070,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="12" spans="1:12" hidden="1" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A12">
         <v>10</v>
       </c>
@@ -1106,7 +1105,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="13" spans="1:12" hidden="1" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A13">
         <v>11</v>
       </c>
@@ -1141,7 +1140,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="14" spans="1:12" hidden="1" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A14">
         <v>12</v>
       </c>
@@ -1176,7 +1175,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="15" spans="1:12" hidden="1" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A15">
         <v>13</v>
       </c>
@@ -1211,7 +1210,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="16" spans="1:12" hidden="1" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A16">
         <v>14</v>
       </c>
@@ -1246,7 +1245,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="17" spans="1:12" hidden="1" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A17">
         <v>15</v>
       </c>
@@ -1281,7 +1280,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="18" spans="1:12" hidden="1" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A18">
         <v>16</v>
       </c>
@@ -1316,7 +1315,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="19" spans="1:12" hidden="1" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A19">
         <v>17</v>
       </c>
@@ -1351,7 +1350,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="20" spans="1:12" hidden="1" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A20">
         <v>18</v>
       </c>
@@ -1386,7 +1385,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="21" spans="1:12" hidden="1" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A21">
         <v>19</v>
       </c>
@@ -1421,7 +1420,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="22" spans="1:12" hidden="1" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A22">
         <v>20</v>
       </c>
@@ -1456,7 +1455,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="23" spans="1:12" hidden="1" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A23">
         <v>21</v>
       </c>
@@ -1476,7 +1475,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="24" spans="1:12" hidden="1" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A24">
         <v>22</v>
       </c>
@@ -1511,7 +1510,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="25" spans="1:12" hidden="1" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A25">
         <v>23</v>
       </c>
@@ -1546,7 +1545,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="26" spans="1:12" hidden="1" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A26">
         <v>24</v>
       </c>
@@ -1581,7 +1580,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="27" spans="1:12" hidden="1" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A27">
         <v>25</v>
       </c>
@@ -1616,7 +1615,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="28" spans="1:12" hidden="1" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A28">
         <v>26</v>
       </c>
@@ -1651,7 +1650,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="29" spans="1:12" hidden="1" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A29">
         <v>27</v>
       </c>
@@ -1686,7 +1685,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="30" spans="1:12" hidden="1" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A30">
         <v>28</v>
       </c>
@@ -1721,7 +1720,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="31" spans="1:12" hidden="1" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A31">
         <v>29</v>
       </c>
@@ -1756,7 +1755,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="32" spans="1:12" hidden="1" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A32">
         <v>30</v>
       </c>
@@ -1791,7 +1790,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="33" spans="1:12" hidden="1" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A33">
         <v>31</v>
       </c>
@@ -1826,7 +1825,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="34" spans="1:12" hidden="1" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A34">
         <v>32</v>
       </c>
@@ -1861,7 +1860,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="35" spans="1:12" hidden="1" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A35">
         <v>33</v>
       </c>
@@ -1922,7 +1921,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="37" spans="1:12" hidden="1" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A37">
         <v>35</v>
       </c>
@@ -2063,7 +2062,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="43" spans="1:12" hidden="1" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:12" x14ac:dyDescent="0.25">
       <c r="H43" t="s">
         <v>41</v>
       </c>
@@ -2080,7 +2079,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="44" spans="1:12" hidden="1" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:12" x14ac:dyDescent="0.25">
       <c r="H44" t="s">
         <v>41</v>
       </c>
@@ -2097,7 +2096,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="45" spans="1:12" hidden="1" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:12" x14ac:dyDescent="0.25">
       <c r="J45">
         <v>19</v>
       </c>
@@ -2108,7 +2107,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="46" spans="1:12" hidden="1" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:12" x14ac:dyDescent="0.25">
       <c r="J46">
         <v>20</v>
       </c>
@@ -2119,7 +2118,7 @@
         <v>81</v>
       </c>
     </row>
-    <row r="47" spans="1:12" hidden="1" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:12" x14ac:dyDescent="0.25">
       <c r="J47">
         <v>21</v>
       </c>
@@ -2130,7 +2129,7 @@
         <v>82</v>
       </c>
     </row>
-    <row r="48" spans="1:12" hidden="1" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:12" x14ac:dyDescent="0.25">
       <c r="J48">
         <v>22</v>
       </c>
@@ -2141,7 +2140,7 @@
         <v>83</v>
       </c>
     </row>
-    <row r="49" spans="10:12" hidden="1" x14ac:dyDescent="0.25">
+    <row r="49" spans="10:12" x14ac:dyDescent="0.25">
       <c r="J49">
         <v>23</v>
       </c>
@@ -2152,7 +2151,7 @@
         <v>84</v>
       </c>
     </row>
-    <row r="50" spans="10:12" hidden="1" x14ac:dyDescent="0.25">
+    <row r="50" spans="10:12" x14ac:dyDescent="0.25">
       <c r="J50">
         <v>24</v>
       </c>
@@ -2163,7 +2162,7 @@
         <v>85</v>
       </c>
     </row>
-    <row r="51" spans="10:12" hidden="1" x14ac:dyDescent="0.25">
+    <row r="51" spans="10:12" x14ac:dyDescent="0.25">
       <c r="J51">
         <v>25</v>
       </c>
@@ -2174,7 +2173,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="52" spans="10:12" hidden="1" x14ac:dyDescent="0.25">
+    <row r="52" spans="10:12" x14ac:dyDescent="0.25">
       <c r="J52">
         <v>26</v>
       </c>
@@ -2185,7 +2184,7 @@
         <v>87</v>
       </c>
     </row>
-    <row r="53" spans="10:12" hidden="1" x14ac:dyDescent="0.25">
+    <row r="53" spans="10:12" x14ac:dyDescent="0.25">
       <c r="J53">
         <v>35</v>
       </c>
@@ -2196,7 +2195,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="54" spans="10:12" hidden="1" x14ac:dyDescent="0.25">
+    <row r="54" spans="10:12" x14ac:dyDescent="0.25">
       <c r="J54">
         <v>36</v>
       </c>
@@ -2207,7 +2206,7 @@
         <v>89</v>
       </c>
     </row>
-    <row r="55" spans="10:12" hidden="1" x14ac:dyDescent="0.25">
+    <row r="55" spans="10:12" x14ac:dyDescent="0.25">
       <c r="J55">
         <v>37</v>
       </c>
@@ -2218,7 +2217,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="56" spans="10:12" hidden="1" x14ac:dyDescent="0.25">
+    <row r="56" spans="10:12" x14ac:dyDescent="0.25">
       <c r="J56">
         <v>38</v>
       </c>
@@ -2229,7 +2228,7 @@
         <v>91</v>
       </c>
     </row>
-    <row r="57" spans="10:12" hidden="1" x14ac:dyDescent="0.25">
+    <row r="57" spans="10:12" x14ac:dyDescent="0.25">
       <c r="J57">
         <v>39</v>
       </c>
@@ -2240,7 +2239,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="58" spans="10:12" hidden="1" x14ac:dyDescent="0.25">
+    <row r="58" spans="10:12" x14ac:dyDescent="0.25">
       <c r="J58">
         <v>40</v>
       </c>
@@ -2251,7 +2250,7 @@
         <v>93</v>
       </c>
     </row>
-    <row r="59" spans="10:12" hidden="1" x14ac:dyDescent="0.25">
+    <row r="59" spans="10:12" x14ac:dyDescent="0.25">
       <c r="J59">
         <v>41</v>
       </c>
@@ -2262,7 +2261,7 @@
         <v>94</v>
       </c>
     </row>
-    <row r="60" spans="10:12" hidden="1" x14ac:dyDescent="0.25">
+    <row r="60" spans="10:12" x14ac:dyDescent="0.25">
       <c r="J60">
         <v>42</v>
       </c>
@@ -2273,7 +2272,7 @@
         <v>95</v>
       </c>
     </row>
-    <row r="61" spans="10:12" hidden="1" x14ac:dyDescent="0.25">
+    <row r="61" spans="10:12" x14ac:dyDescent="0.25">
       <c r="J61">
         <v>43</v>
       </c>
@@ -2284,7 +2283,7 @@
         <v>96</v>
       </c>
     </row>
-    <row r="62" spans="10:12" hidden="1" x14ac:dyDescent="0.25">
+    <row r="62" spans="10:12" x14ac:dyDescent="0.25">
       <c r="J62">
         <v>44</v>
       </c>
@@ -2295,7 +2294,7 @@
         <v>97</v>
       </c>
     </row>
-    <row r="63" spans="10:12" hidden="1" x14ac:dyDescent="0.25">
+    <row r="63" spans="10:12" x14ac:dyDescent="0.25">
       <c r="J63">
         <v>45</v>
       </c>
@@ -2306,7 +2305,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="64" spans="10:12" hidden="1" x14ac:dyDescent="0.25">
+    <row r="64" spans="10:12" x14ac:dyDescent="0.25">
       <c r="J64">
         <v>46</v>
       </c>
@@ -2317,7 +2316,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="65" spans="8:12" hidden="1" x14ac:dyDescent="0.25">
+    <row r="65" spans="8:12" x14ac:dyDescent="0.25">
       <c r="J65">
         <v>47</v>
       </c>
@@ -2328,7 +2327,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="66" spans="8:12" hidden="1" x14ac:dyDescent="0.25">
+    <row r="66" spans="8:12" x14ac:dyDescent="0.25">
       <c r="J66">
         <v>48</v>
       </c>
@@ -2339,7 +2338,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="67" spans="8:12" hidden="1" x14ac:dyDescent="0.25">
+    <row r="67" spans="8:12" x14ac:dyDescent="0.25">
       <c r="H67" t="s">
         <v>46</v>
       </c>
@@ -2356,7 +2355,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="68" spans="8:12" hidden="1" x14ac:dyDescent="0.25">
+    <row r="68" spans="8:12" x14ac:dyDescent="0.25">
       <c r="H68" t="s">
         <v>46</v>
       </c>
@@ -2373,7 +2372,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="69" spans="8:12" hidden="1" x14ac:dyDescent="0.25">
+    <row r="69" spans="8:12" x14ac:dyDescent="0.25">
       <c r="H69" t="s">
         <v>46</v>
       </c>
@@ -2390,7 +2389,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="70" spans="8:12" hidden="1" x14ac:dyDescent="0.25">
+    <row r="70" spans="8:12" x14ac:dyDescent="0.25">
       <c r="H70" t="s">
         <v>46</v>
       </c>
@@ -2407,7 +2406,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="71" spans="8:12" hidden="1" x14ac:dyDescent="0.25">
+    <row r="71" spans="8:12" x14ac:dyDescent="0.25">
       <c r="H71" t="s">
         <v>46</v>
       </c>
@@ -2424,7 +2423,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="72" spans="8:12" hidden="1" x14ac:dyDescent="0.25">
+    <row r="72" spans="8:12" x14ac:dyDescent="0.25">
       <c r="H72" t="s">
         <v>46</v>
       </c>
@@ -2441,7 +2440,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="73" spans="8:12" hidden="1" x14ac:dyDescent="0.25">
+    <row r="73" spans="8:12" x14ac:dyDescent="0.25">
       <c r="H73" t="s">
         <v>46</v>
       </c>
@@ -2458,7 +2457,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="74" spans="8:12" hidden="1" x14ac:dyDescent="0.25">
+    <row r="74" spans="8:12" x14ac:dyDescent="0.25">
       <c r="H74" t="s">
         <v>46</v>
       </c>
@@ -2475,7 +2474,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="75" spans="8:12" hidden="1" x14ac:dyDescent="0.25">
+    <row r="75" spans="8:12" x14ac:dyDescent="0.25">
       <c r="H75" t="s">
         <v>41</v>
       </c>
@@ -2492,7 +2491,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="76" spans="8:12" hidden="1" x14ac:dyDescent="0.25">
+    <row r="76" spans="8:12" x14ac:dyDescent="0.25">
       <c r="H76" t="s">
         <v>41</v>
       </c>
@@ -2509,7 +2508,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="77" spans="8:12" hidden="1" x14ac:dyDescent="0.25">
+    <row r="77" spans="8:12" x14ac:dyDescent="0.25">
       <c r="J77">
         <v>59</v>
       </c>
@@ -2520,7 +2519,7 @@
         <v>102</v>
       </c>
     </row>
-    <row r="78" spans="8:12" hidden="1" x14ac:dyDescent="0.25">
+    <row r="78" spans="8:12" x14ac:dyDescent="0.25">
       <c r="J78">
         <v>60</v>
       </c>
@@ -2531,7 +2530,7 @@
         <v>103</v>
       </c>
     </row>
-    <row r="79" spans="8:12" hidden="1" x14ac:dyDescent="0.25">
+    <row r="79" spans="8:12" x14ac:dyDescent="0.25">
       <c r="J79">
         <v>61</v>
       </c>
@@ -2542,7 +2541,7 @@
         <v>104</v>
       </c>
     </row>
-    <row r="80" spans="8:12" hidden="1" x14ac:dyDescent="0.25">
+    <row r="80" spans="8:12" x14ac:dyDescent="0.25">
       <c r="J80">
         <v>62</v>
       </c>
@@ -2553,7 +2552,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="81" spans="8:12" hidden="1" x14ac:dyDescent="0.25">
+    <row r="81" spans="8:12" x14ac:dyDescent="0.25">
       <c r="J81">
         <v>63</v>
       </c>
@@ -2564,7 +2563,7 @@
         <v>106</v>
       </c>
     </row>
-    <row r="82" spans="8:12" hidden="1" x14ac:dyDescent="0.25">
+    <row r="82" spans="8:12" x14ac:dyDescent="0.25">
       <c r="J82">
         <v>64</v>
       </c>
@@ -2575,7 +2574,7 @@
         <v>107</v>
       </c>
     </row>
-    <row r="83" spans="8:12" hidden="1" x14ac:dyDescent="0.25">
+    <row r="83" spans="8:12" x14ac:dyDescent="0.25">
       <c r="J83">
         <v>65</v>
       </c>
@@ -2586,7 +2585,7 @@
         <v>108</v>
       </c>
     </row>
-    <row r="84" spans="8:12" hidden="1" x14ac:dyDescent="0.25">
+    <row r="84" spans="8:12" x14ac:dyDescent="0.25">
       <c r="J84">
         <v>66</v>
       </c>
@@ -2597,7 +2596,7 @@
         <v>109</v>
       </c>
     </row>
-    <row r="85" spans="8:12" hidden="1" x14ac:dyDescent="0.25">
+    <row r="85" spans="8:12" x14ac:dyDescent="0.25">
       <c r="H85" t="s">
         <v>42</v>
       </c>
@@ -2614,7 +2613,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="86" spans="8:12" hidden="1" x14ac:dyDescent="0.25">
+    <row r="86" spans="8:12" x14ac:dyDescent="0.25">
       <c r="H86" t="s">
         <v>42</v>
       </c>
@@ -2631,7 +2630,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="87" spans="8:12" hidden="1" x14ac:dyDescent="0.25">
+    <row r="87" spans="8:12" x14ac:dyDescent="0.25">
       <c r="H87" t="s">
         <v>42</v>
       </c>
@@ -2648,7 +2647,7 @@
         <v>63</v>
       </c>
     </row>
-    <row r="88" spans="8:12" hidden="1" x14ac:dyDescent="0.25">
+    <row r="88" spans="8:12" x14ac:dyDescent="0.25">
       <c r="H88" t="s">
         <v>42</v>
       </c>
@@ -2665,7 +2664,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="89" spans="8:12" hidden="1" x14ac:dyDescent="0.25">
+    <row r="89" spans="8:12" x14ac:dyDescent="0.25">
       <c r="H89" t="s">
         <v>42</v>
       </c>
@@ -2682,7 +2681,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="90" spans="8:12" hidden="1" x14ac:dyDescent="0.25">
+    <row r="90" spans="8:12" x14ac:dyDescent="0.25">
       <c r="H90" t="s">
         <v>42</v>
       </c>
@@ -2699,7 +2698,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="91" spans="8:12" hidden="1" x14ac:dyDescent="0.25">
+    <row r="91" spans="8:12" x14ac:dyDescent="0.25">
       <c r="H91" t="s">
         <v>42</v>
       </c>
@@ -2716,7 +2715,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="92" spans="8:12" hidden="1" x14ac:dyDescent="0.25">
+    <row r="92" spans="8:12" x14ac:dyDescent="0.25">
       <c r="H92" t="s">
         <v>42</v>
       </c>
@@ -2733,7 +2732,7 @@
         <v>68</v>
       </c>
     </row>
-    <row r="93" spans="8:12" hidden="1" x14ac:dyDescent="0.25">
+    <row r="93" spans="8:12" x14ac:dyDescent="0.25">
       <c r="J93">
         <v>75</v>
       </c>
@@ -2744,7 +2743,7 @@
         <v>110</v>
       </c>
     </row>
-    <row r="94" spans="8:12" hidden="1" x14ac:dyDescent="0.25">
+    <row r="94" spans="8:12" x14ac:dyDescent="0.25">
       <c r="J94">
         <v>76</v>
       </c>
@@ -2755,7 +2754,7 @@
         <v>111</v>
       </c>
     </row>
-    <row r="95" spans="8:12" hidden="1" x14ac:dyDescent="0.25">
+    <row r="95" spans="8:12" x14ac:dyDescent="0.25">
       <c r="J95">
         <v>77</v>
       </c>
@@ -2766,7 +2765,7 @@
         <v>112</v>
       </c>
     </row>
-    <row r="96" spans="8:12" hidden="1" x14ac:dyDescent="0.25">
+    <row r="96" spans="8:12" x14ac:dyDescent="0.25">
       <c r="J96">
         <v>78</v>
       </c>
@@ -2777,7 +2776,7 @@
         <v>113</v>
       </c>
     </row>
-    <row r="97" spans="8:12" hidden="1" x14ac:dyDescent="0.25">
+    <row r="97" spans="8:12" x14ac:dyDescent="0.25">
       <c r="J97">
         <v>79</v>
       </c>
@@ -2788,7 +2787,7 @@
         <v>114</v>
       </c>
     </row>
-    <row r="98" spans="8:12" hidden="1" x14ac:dyDescent="0.25">
+    <row r="98" spans="8:12" x14ac:dyDescent="0.25">
       <c r="J98">
         <v>80</v>
       </c>
@@ -2799,7 +2798,7 @@
         <v>115</v>
       </c>
     </row>
-    <row r="99" spans="8:12" hidden="1" x14ac:dyDescent="0.25">
+    <row r="99" spans="8:12" x14ac:dyDescent="0.25">
       <c r="H99" t="s">
         <v>41</v>
       </c>
@@ -2808,7 +2807,7 @@
       </c>
       <c r="K99" s="1"/>
     </row>
-    <row r="100" spans="8:12" hidden="1" x14ac:dyDescent="0.25">
+    <row r="100" spans="8:12" x14ac:dyDescent="0.25">
       <c r="H100" t="s">
         <v>41</v>
       </c>
@@ -2817,7 +2816,7 @@
       </c>
       <c r="K100" s="1"/>
     </row>
-    <row r="101" spans="8:12" hidden="1" x14ac:dyDescent="0.25">
+    <row r="101" spans="8:12" x14ac:dyDescent="0.25">
       <c r="H101" t="s">
         <v>69</v>
       </c>
@@ -2825,7 +2824,7 @@
         <v>70</v>
       </c>
     </row>
-    <row r="102" spans="8:12" hidden="1" x14ac:dyDescent="0.25">
+    <row r="102" spans="8:12" x14ac:dyDescent="0.25">
       <c r="H102" t="s">
         <v>69</v>
       </c>
@@ -2833,7 +2832,7 @@
         <v>71</v>
       </c>
     </row>
-    <row r="103" spans="8:12" hidden="1" x14ac:dyDescent="0.25">
+    <row r="103" spans="8:12" x14ac:dyDescent="0.25">
       <c r="H103" t="s">
         <v>69</v>
       </c>
@@ -2841,7 +2840,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="104" spans="8:12" hidden="1" x14ac:dyDescent="0.25">
+    <row r="104" spans="8:12" x14ac:dyDescent="0.25">
       <c r="H104" t="s">
         <v>69</v>
       </c>
@@ -2849,7 +2848,7 @@
         <v>73</v>
       </c>
     </row>
-    <row r="105" spans="8:12" hidden="1" x14ac:dyDescent="0.25">
+    <row r="105" spans="8:12" x14ac:dyDescent="0.25">
       <c r="H105" t="s">
         <v>69</v>
       </c>
@@ -2857,7 +2856,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="106" spans="8:12" hidden="1" x14ac:dyDescent="0.25">
+    <row r="106" spans="8:12" x14ac:dyDescent="0.25">
       <c r="H106" t="s">
         <v>69</v>
       </c>
@@ -2865,7 +2864,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="107" spans="8:12" hidden="1" x14ac:dyDescent="0.25">
+    <row r="107" spans="8:12" x14ac:dyDescent="0.25">
       <c r="H107" t="s">
         <v>69</v>
       </c>
@@ -2873,7 +2872,7 @@
         <v>76</v>
       </c>
     </row>
-    <row r="108" spans="8:12" hidden="1" x14ac:dyDescent="0.25">
+    <row r="108" spans="8:12" x14ac:dyDescent="0.25">
       <c r="H108" t="s">
         <v>69</v>
       </c>
@@ -2882,13 +2881,7 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A2:L108" xr:uid="{CF3C1C7E-605D-41A8-B4C8-47EE79D051C7}">
-    <filterColumn colId="4">
-      <filters>
-        <filter val="Control"/>
-      </filters>
-    </filterColumn>
-  </autoFilter>
+  <autoFilter ref="A2:L108" xr:uid="{CF3C1C7E-605D-41A8-B4C8-47EE79D051C7}"/>
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A3:C47">
     <sortCondition ref="C3:C47"/>
   </sortState>

</xml_diff>